<commit_message>
Fix building-to-upload pairing when workbook file_name differs
Pair uploads to Buildings sheet rows by order when file_name does not
match the uploaded filename. Show warnings in the app, reject empty
uploads, and skip blank zero-value manual template rows.

Co-authored-by: Tom <tsgwilliam@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/apps/oneclick/templates/Etude_OneClick_Project.xlsx
+++ b/apps/oneclick/templates/Etude_OneClick_Project.xlsx
@@ -443,12 +443,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>example_detailReport.xls</t>
+          <t>detailReport_example.xls</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Example building</t>
+          <t>Building 1</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -512,7 +512,11 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Building 1</t>
+        </is>
+      </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>A1-A3</t>
@@ -532,7 +536,11 @@
         <v>0</v>
       </c>
       <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Set kgCO2e/m2 and building name, or leave blank to skip</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Reject summary exports; pre-fill project workbook from uploads
Validate detailReport uploads by checking for a Section header row.
Pre-populate the downloadable project workbook Buildings sheet with
exact filenames from files already in the OneClick upload box, preserving
any GIA or names from an existing project workbook when re-downloading.

Co-authored-by: Tom <tsgwilliam@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/apps/oneclick/templates/Etude_OneClick_Project.xlsx
+++ b/apps/oneclick/templates/Etude_OneClick_Project.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,37 +508,6 @@
       <c r="G1" t="inlineStr">
         <is>
           <t>notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Building 1</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>A1-A3</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>5.3</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Manual benchmark example</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Set kgCO2e/m2 and building name, or leave blank to skip</t>
         </is>
       </c>
     </row>

</xml_diff>